<commit_message>
Updated test cases, Description and Outcome Message text.
</commit_message>
<xml_diff>
--- a/rules/CORE-000457/positive/01/data/unit-test-coreid-CG0373-positive.xlsx
+++ b/rules/CORE-000457/positive/01/data/unit-test-coreid-CG0373-positive.xlsx
@@ -21,9 +21,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -130,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -171,10 +170,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1342,378 +1342,516 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>STUDYID</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>DOMAIN</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>USUBJID</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>ECSEQ</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>ECLNKID</t>
+        </is>
+      </c>
+      <c r="F1" s="13" t="inlineStr">
+        <is>
+          <t>ECTRT</t>
+        </is>
+      </c>
+      <c r="G1" s="13" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+      <c r="H1" s="13" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="I1" s="13" t="inlineStr">
+        <is>
+          <t>ECREASOC</t>
+        </is>
+      </c>
+      <c r="J1" s="13" t="inlineStr">
+        <is>
+          <t>ECDOSE</t>
+        </is>
+      </c>
+      <c r="K1" s="13" t="inlineStr">
+        <is>
+          <t>ECDOSTXT</t>
+        </is>
+      </c>
+      <c r="L1" s="13" t="inlineStr">
+        <is>
+          <t>ECDOSU</t>
+        </is>
+      </c>
+      <c r="M1" s="13" t="inlineStr">
+        <is>
+          <t>ECDOSFRM</t>
+        </is>
+      </c>
+      <c r="N1" s="13" t="inlineStr">
+        <is>
+          <t>ECSTDTC</t>
+        </is>
+      </c>
+      <c r="O1" s="13" t="inlineStr">
+        <is>
+          <t>ECENDTC</t>
+        </is>
+      </c>
+      <c r="P1" s="13" t="inlineStr">
+        <is>
+          <t>ECSTDY</t>
+        </is>
+      </c>
+      <c r="Q1" s="13" t="inlineStr">
+        <is>
+          <t>ECENDY</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="n"/>
-      <c r="B2" s="12" t="n"/>
-      <c r="C2" s="12" t="n"/>
-      <c r="D2" s="12" t="n"/>
-      <c r="E2" s="12" t="n"/>
-      <c r="F2" s="12" t="n"/>
-      <c r="G2" s="12" t="n"/>
-      <c r="H2" s="12" t="n"/>
-      <c r="I2" s="12" t="n"/>
-      <c r="J2" s="12" t="n"/>
-      <c r="K2" s="12" t="n"/>
-      <c r="L2" s="12" t="n"/>
-      <c r="M2" s="12" t="n"/>
-      <c r="N2" s="12" t="n"/>
-      <c r="O2" s="12" t="n"/>
-      <c r="P2" s="12" t="n"/>
-      <c r="Q2" s="12" t="n"/>
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Study Identifier</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>Domain Abbreviation</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>Unique Subject Identifier</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>Sequence Number</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Link ID</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Name of Treatment</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>Pre-Specified</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>Occurrence</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>Reason for Occur Value</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>Dose</t>
+        </is>
+      </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>Dose Description</t>
+        </is>
+      </c>
+      <c r="L2" s="14" t="inlineStr">
+        <is>
+          <t>Dose Units</t>
+        </is>
+      </c>
+      <c r="M2" s="14" t="inlineStr">
+        <is>
+          <t>Dose Form</t>
+        </is>
+      </c>
+      <c r="N2" s="14" t="inlineStr">
+        <is>
+          <t>Start Date/Time of Treatment</t>
+        </is>
+      </c>
+      <c r="O2" s="14" t="inlineStr">
+        <is>
+          <t>End Date/Time of Treatment</t>
+        </is>
+      </c>
+      <c r="P2" s="14" t="inlineStr">
+        <is>
+          <t>Study Day of Start of Treatment</t>
+        </is>
+      </c>
+      <c r="Q2" s="14" t="inlineStr">
+        <is>
+          <t>Study Day of End of Treatment</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="n"/>
-      <c r="B3" s="12" t="n"/>
-      <c r="C3" s="12" t="n"/>
-      <c r="D3" s="12" t="n"/>
-      <c r="E3" s="12" t="n"/>
-      <c r="F3" s="12" t="n"/>
-      <c r="G3" s="12" t="n"/>
-      <c r="H3" s="12" t="n"/>
-      <c r="I3" s="12" t="n"/>
-      <c r="J3" s="12" t="n"/>
-      <c r="K3" s="12" t="n"/>
-      <c r="L3" s="12" t="n"/>
-      <c r="M3" s="12" t="n"/>
-      <c r="N3" s="12" t="n"/>
-      <c r="O3" s="12" t="n"/>
-      <c r="P3" s="12" t="n"/>
-      <c r="Q3" s="12" t="n"/>
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="K3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="L3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="M3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="N3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="O3" s="14" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="P3" s="14" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q3" s="14" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>STUDYID</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>USUBJID</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>ECSEQ</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>ECLNKID</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>ECTRT</t>
-        </is>
-      </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>ECPRESP</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>ECOCCUR</t>
-        </is>
-      </c>
-      <c r="I4" s="13" t="inlineStr">
-        <is>
-          <t>ECREASOC</t>
-        </is>
-      </c>
-      <c r="J4" s="13" t="inlineStr">
-        <is>
-          <t>ECDOSE</t>
-        </is>
-      </c>
-      <c r="K4" s="13" t="inlineStr">
-        <is>
-          <t>ECDOSTXT</t>
-        </is>
-      </c>
-      <c r="L4" s="13" t="inlineStr">
-        <is>
-          <t>ECDOSU</t>
-        </is>
-      </c>
-      <c r="M4" s="13" t="inlineStr">
-        <is>
-          <t>ECDOSFRM</t>
-        </is>
-      </c>
-      <c r="N4" s="13" t="inlineStr">
-        <is>
-          <t>ECSTDTC</t>
-        </is>
-      </c>
-      <c r="O4" s="13" t="inlineStr">
-        <is>
-          <t>ECENDTC</t>
-        </is>
-      </c>
-      <c r="P4" s="13" t="inlineStr">
-        <is>
-          <t>ECSTDY</t>
-        </is>
-      </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>ECENDY</t>
-        </is>
+      <c r="A4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="M4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="N4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="O4" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="P4" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="14" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>Study Identifier</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Domain Abbreviation</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>Unique Subject Identifier</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>Sequence Number</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>Link ID</t>
-        </is>
-      </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>Name of Treatment</t>
-        </is>
-      </c>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>Pre-Specified</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr">
-        <is>
-          <t>Occurrence</t>
-        </is>
-      </c>
-      <c r="I5" s="14" t="inlineStr">
-        <is>
-          <t>Reason for Occur Value</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="inlineStr">
-        <is>
-          <t>Dose</t>
-        </is>
-      </c>
-      <c r="K5" s="14" t="inlineStr">
-        <is>
-          <t>Dose Description</t>
-        </is>
-      </c>
-      <c r="L5" s="14" t="inlineStr">
-        <is>
-          <t>Dose Units</t>
-        </is>
-      </c>
-      <c r="M5" s="14" t="inlineStr">
-        <is>
-          <t>Dose Form</t>
-        </is>
-      </c>
-      <c r="N5" s="14" t="inlineStr">
-        <is>
-          <t>Start Date/Time of Treatment</t>
-        </is>
-      </c>
-      <c r="O5" s="14" t="inlineStr">
-        <is>
-          <t>End Date/Time of Treatment</t>
-        </is>
-      </c>
-      <c r="P5" s="14" t="inlineStr">
-        <is>
-          <t>Study Day of Start of Treatment</t>
-        </is>
-      </c>
-      <c r="Q5" s="14" t="inlineStr">
-        <is>
-          <t>Study Day of End of Treatment</t>
-        </is>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ABC1001</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A2-20110114</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>BOTTLE A</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="15" t="n"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>TABLET</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>QD</t>
+        </is>
+      </c>
+      <c r="N5" s="18" t="n">
+        <v>40557</v>
+      </c>
+      <c r="O5" s="18" t="n">
+        <v>40571</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>Num</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>Num</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="L6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="M6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="N6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="O6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="P6" s="14" t="inlineStr">
-        <is>
-          <t>Num</t>
-        </is>
-      </c>
-      <c r="Q6" s="14" t="inlineStr">
-        <is>
-          <t>Num</t>
-        </is>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ABC2001</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A2-20110114</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>BOTTLE A</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="15" t="n"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>QD</t>
+        </is>
+      </c>
+      <c r="N6" s="18" t="n">
+        <v>40557</v>
+      </c>
+      <c r="O6" s="18" t="n">
+        <v>40566</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="B7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="C7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="D7" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="G7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="H7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="I7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="J7" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="L7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="M7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="N7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="O7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="P7" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q7" s="14" t="n">
-        <v>8</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ABC2001</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A0-20110124</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BOTTLE A</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>PATIENT MISTAKE</t>
+        </is>
+      </c>
+      <c r="K7" s="15" t="n"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>TABLET</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>QD</t>
+        </is>
+      </c>
+      <c r="N7" s="18" t="n">
+        <v>40567</v>
+      </c>
+      <c r="O7" s="18" t="n">
+        <v>40567</v>
+      </c>
+      <c r="P7" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -1729,15 +1867,15 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ABC1001</t>
+          <t>ABC2001</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>A2-20110114</t>
+          <t>A2-20110125</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1769,211 +1907,16 @@
           <t>QD</t>
         </is>
       </c>
-      <c r="N8" s="16" t="n">
-        <v>40557</v>
-      </c>
-      <c r="O8" s="16" t="n">
+      <c r="N8" s="18" t="n">
+        <v>40568</v>
+      </c>
+      <c r="O8" s="18" t="n">
         <v>40571</v>
       </c>
       <c r="P8" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="Q8" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ABC</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>ABC2001</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>A2-20110114</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>BOTTLE A</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" s="15" t="n"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>QD</t>
-        </is>
-      </c>
-      <c r="N9" s="16" t="n">
-        <v>40557</v>
-      </c>
-      <c r="O9" s="16" t="n">
-        <v>40566</v>
-      </c>
-      <c r="P9" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ABC</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>ABC2001</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>A0-20110124</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>BOTTLE A</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>PATIENT MISTAKE</t>
-        </is>
-      </c>
-      <c r="K10" s="15" t="n"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>TABLET</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>QD</t>
-        </is>
-      </c>
-      <c r="N10" s="16" t="n">
-        <v>40567</v>
-      </c>
-      <c r="O10" s="16" t="n">
-        <v>40567</v>
-      </c>
-      <c r="P10" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ABC</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>ABC2001</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>A2-20110125</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>BOTTLE A</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>2</v>
-      </c>
-      <c r="K11" s="15" t="n"/>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>TABLET</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>QD</t>
-        </is>
-      </c>
-      <c r="N11" s="16" t="n">
-        <v>40568</v>
-      </c>
-      <c r="O11" s="16" t="n">
-        <v>40571</v>
-      </c>
-      <c r="P11" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q11" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>